<commit_message>
Unilever run: bear case at 3.45% Bund
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/ULVR/2026-10-14/bear/scratch/00_control/out/dcf.xlsx
+++ b/runs/ULVR/2026-10-14/bear/scratch/00_control/out/dcf.xlsx
@@ -584,11 +584,11 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.0318</v>
+        <v>0.0345</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FRED IRLTLT01DEM156N (German 10-year Bund yield, OECD monthly average), latest month 2026-08-01 (Aug 2026 average 3.18%); PM decision 7: euro cash flows -&gt; Bund, not the gilt.</t>
+          <t>PM decision 14 Oct 2026 (decision 11; briefs/ULVR.yaml wacc.risk_free comment; docs/phase5/ulvr-evidence-audit.md): German 10-year Bund yield on the run date, 3.45% on 14 Oct 2026 (Trading Economics https://tradingeconomics.com/germany/government-bond-yield; also Bloomberg rates page https://www.bloomberg.com/markets/rates-bonds); cross-check 3.50% on 9 Oct 2026 (https://www.thetrading.tools/germany-10-year-yield). Replaces FRED IRLTLT01DEM156N (OECD monthly average, latest Aug 2026 = 3.18%, two months old). FLAG: data aggregator, not a primary source; the Bundesbank and ECB daily series (and these aggregator pages) are blocked from the Data agent's environment, so the Data agent could not re-check the 3.45% figure itself (PM-supplied, from the evidence audit).</t>
         </is>
       </c>
     </row>
@@ -629,11 +629,11 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.0388</v>
+        <v>0.0415</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>risk-free 3.18% + credit spread 0.70% (PM rule, briefs)</t>
+          <t>risk-free 3.45% + credit spread 0.70% (PM rule, briefs)</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,11 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7228.7</v>
+        <v>7061.8</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PM decision 14 Oct 2026 (decision 10, docs/phase5/ulvr-run-flags.md item B, C, D; E agreed 13 Oct; briefs/ULVR.yaml comments): sum of (1) TMICC 19.85%: 121,604,413 shares (TMICC resale prospectus, Form 424(b)(4) (accession 0001104659-26-042683, 13 Apr 2026)) x EUR 15.914 (Yahoo MICC.AS close 2026-10-13) = 1,935.2; (2) joint ventures by Gordon growth: FY25 dividends received from JVs and associates EUR 229m (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11: JVs 'Dividends received/reductions (229)', associates nil; the p.132 cash-flow line is 243 because it also includes dividends from other non-current investments, which are valued in (4)) x (1 + 1.6%) / (cost of equity 7.6020% - 1.6%) = 3,876.4, cost of equity = risk-free 3.18% (inputs.yaml) + beta 0.8844 (inputs.yaml, Risk agent) x ERP 5.0% (brief); (3) associates at book 15 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11); (4) other fair-value financial investments 902 = equity investments FVOCI excl. TMICC 561 (2,216 - 1,655) + non-current FVTPL 'Other' 341 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.174 note 17A); amortised-cost assets 368 (incl. judicial deposits 175) excluded; (5) net Magnum transition balance owed to Unilever 2,100 - 1,600 = 500 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) notes 13-14, p.159-160). Was 2,044.2 (TMICC + JVs/associates at book 109). If the run's cost of equity changes, the JV value must be recomputed.</t>
+          <t>PM decision 14 Oct 2026 (decision 10, docs/phase5/ulvr-run-flags.md item B, C, D; E agreed 13 Oct; briefs/ULVR.yaml comments): sum of (1) TMICC 19.85%: 121,604,413 shares (TMICC resale prospectus, Form 424(b)(4) (accession 0001104659-26-042683, 13 Apr 2026)) x EUR 15.914 (Yahoo MICC.AS close 2026-10-13) = 1,935.2; (2) joint ventures by Gordon growth: FY25 dividends received from JVs and associates EUR 229m (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11: JVs 'Dividends received/reductions (229)', associates nil; the p.132 cash-flow line is 243 because it also includes dividends from other non-current investments, which are valued in (4)) x (1 + 1.6%) / (cost of equity 7.8720% - 1.6%) = 3,709.6, cost of equity = risk-free 3.45% (inputs.yaml) + beta 0.8844 (inputs.yaml, Risk agent) x ERP 5.0% (brief); (3) associates at book 15 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11); (4) other fair-value financial investments 902 = equity investments FVOCI excl. TMICC 561 (2,216 - 1,655) + non-current FVTPL 'Other' 341 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.174 note 17A); amortised-cost assets 368 (incl. judicial deposits 175) excluded; (5) net Magnum transition balance owed to Unilever 2,100 - 1,600 = 500 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) notes 13-14, p.159-160). Was 2,044.2 (TMICC + JVs/associates at book 109). If the run's cost of equity changes, the JV value must be recomputed.</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>4031.190822495119</v>
+        <v>3987.561070822048</v>
       </c>
     </row>
     <row r="16">
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.07602</v>
+        <v>0.07872000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1408,7 +1408,7 @@
         <v/>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.028712</v>
+        <v>0.03071</v>
       </c>
     </row>
     <row r="19">
@@ -1422,7 +1422,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.0683868542</v>
+        <v>0.0709735865</v>
       </c>
     </row>
     <row r="20">
@@ -1436,7 +1436,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>22294.53449265338</v>
+        <v>22165.44187139205</v>
       </c>
     </row>
     <row r="21">
@@ -1464,7 +1464,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>98543.52340345255</v>
+        <v>93906.64720212416</v>
       </c>
     </row>
     <row r="23">
@@ -1478,7 +1478,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>73172.80032233591</v>
+        <v>68975.03274216867</v>
       </c>
     </row>
     <row r="24">
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>95467.33481498928</v>
+        <v>91140.47461356071</v>
       </c>
     </row>
     <row r="25">
@@ -1506,7 +1506,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10199.73005163346</v>
+        <v>9737.448307712826</v>
       </c>
     </row>
     <row r="26">
@@ -1520,7 +1520,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>102875.6047633558</v>
+        <v>98844.12630584789</v>
       </c>
     </row>
     <row r="27">
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>102302.2443212835</v>
+        <v>98163.22535806705</v>
       </c>
     </row>
     <row r="28">
@@ -1548,7 +1548,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>47.48685544578252</v>
+        <v>45.56559754476966</v>
       </c>
     </row>
     <row r="29">
@@ -1562,7 +1562,7 @@
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>4017.842414427726</v>
+        <v>3855.285609786128</v>
       </c>
     </row>
     <row r="30">
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>-0.1470454486</v>
+        <v>-0.1815549072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unilever bear re-run in progress
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/ULVR/2026-10-14/bear/scratch/00_control/out/dcf.xlsx
+++ b/runs/ULVR/2026-10-14/bear/scratch/00_control/out/dcf.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.03965993983898081</v>
+        <v>0.0396599398389808</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.05</v>
+        <v>0.042</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -734,11 +734,11 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>35890.5</v>
+        <v>35247.6</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bridge items already at run-date market prices (not grown in the roll-forward; mistakes log row 24): TMICC stake 1,935.2 (inputs.yaml `associates` component (1): 121,604,413 shares x EUR 15.914, Yahoo MICC.AS close 2026-10-13) + Foods consideration 33,955.3 (inputs.yaml `disposal_proceeds`: USD 15,700m cash + 499,691,175 McCormick shares x USD 44.64, Yahoo MKC close 2026-10-13, at FRED DEXUSEU) = 35,890.5. Excluded (balance-sheet-date values): JVs by Gordon growth on FY25 dividends, associates at book 15, fair-value investments 902 (31 Dec 2025), Magnum transition balance 500.</t>
+          <t>Bridge items already at run-date market prices (not grown in the roll-forward; mistakes log row 24): TMICC stake 1,935.2 (inputs.yaml `associates` component (1): 121,604,413 shares x EUR 15.914, Yahoo MICC.AS close 2026-10-13) + Foods consideration 33,955.3 (inputs.yaml `disposal_proceeds`: USD 15,700m cash + 499,691,175 McCormick shares x USD 44.64, Yahoo MKC close 2026-10-13, at FRED DEXUSEU) = 35,890.5. Excluded (balance-sheet-date values): JVs by Gordon growth on FY25 dividends, associates at book 15, fair-value investments 902 (31 Dec 2025), Magnum transition balance 500. LESS McCormick dividends the new shares miss before closing (PM decision 15 Oct 2026): 499,691,175 shares x USD 0.48 a quarter (McCormick 10-Q to 31 Aug 2026, accession 0000063754-26-000329) x 3 quarters (ex-dates Jan, Apr, Jul 2027; closing expected mid-2027, Form 425 0000217410-26-000027) / 1.1193 USD per EUR (FRED DEXUSEU 2026-10-09) = 642.9; 35890.5 - 642.9. FLAG: if closing comes before the July ex-date, 2 quarters (+c.8p)</t>
         </is>
       </c>
     </row>
@@ -809,11 +809,11 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0</v>
+        <v>698.6</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Brief rule (0 if in surplus): net SURPLUS EUR 3,518m at 31 Dec 2025 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.43 and note 4B; XBRL ifrs-full:LiabilityAssetOfDefinedBenefitPlans = -3,518); gross deficit plans 944 (funded in deficit 100 + unfunded 844, p.131) are inside that net figure. 30 Jun 2026: surplus 3.7bn (Unilever H1 2026 results 6-K (accession 0000217410-26-000057, 28 Jul 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000057/ul-20260630.htm)).</t>
+          <t>PM decision 15 Oct 2026 (evidence audit): plans in deficit 944 (funded in deficit 100 + unfunded 844, Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026) p.131) x (1 - 26% tax, briefs/ULVR.yaml tax_rate) = 698.6. The net surplus (3,518) is not offset against them; surpluses are not added (brief rule)</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,11 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7061.8</v>
+        <v>7533.5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PM decision 14 Oct 2026 (decision 10, docs/phase5/ulvr-run-flags.md item B, C, D; E agreed 13 Oct; briefs/ULVR.yaml comments): sum of (1) TMICC 19.85%: 121,604,413 shares (TMICC resale prospectus, Form 424(b)(4) (accession 0001104659-26-042683, 13 Apr 2026)) x EUR 15.914 (Yahoo MICC.AS close 2026-10-13) = 1,935.2; (2) joint ventures by Gordon growth: FY25 dividends received from JVs and associates EUR 229m (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11: JVs 'Dividends received/reductions (229)', associates nil; the p.132 cash-flow line is 243 because it also includes dividends from other non-current investments, which are valued in (4)) x (1 + 1.6%) / (cost of equity 7.8720% - 1.6%) = 3,709.6, cost of equity = risk-free 3.45% (inputs.yaml) + beta 0.8844 (inputs.yaml, Risk agent) x ERP 5.0% (brief); (3) associates at book 15 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11); (4) other fair-value financial investments 902 = equity investments FVOCI excl. TMICC 561 (2,216 - 1,655) + non-current FVTPL 'Other' 341 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.174 note 17A); amortised-cost assets 368 (incl. judicial deposits 175) excluded; (5) net Magnum transition balance owed to Unilever 2,100 - 1,600 = 500 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) notes 13-14, p.159-160). Was 2,044.2 (TMICC + JVs/associates at book 109). If the run's cost of equity changes, the JV value must be recomputed.</t>
+          <t>PM decision 14 Oct 2026 (decision 10, docs/phase5/ulvr-run-flags.md item B, C, D; E agreed 13 Oct; briefs/ULVR.yaml comments): sum of (1) TMICC 19.85%: 121,604,413 shares (TMICC resale prospectus, Form 424(b)(4) (accession 0001104659-26-042683, 13 Apr 2026)) x EUR 15.914 (Yahoo MICC.AS close 2026-10-13) = 1,935.2; (2) joint ventures by Gordon growth: FY25 dividends received from JVs and associates EUR 229m (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11: JVs 'Dividends received/reductions (229)', associates nil; the p.132 cash-flow line is 243 because it also includes dividends from other non-current investments, which are valued in (4)) x (1 + 1.6%) / (cost of equity 7.8720% - 1.6%) = 3,709.6, cost of equity = risk-free 3.45% (inputs.yaml) + beta 0.8844 (inputs.yaml, Risk agent) x ERP 5.0% (brief); (3) associates at book 15 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.158 note 11); (4) other fair-value financial investments 902 = equity investments FVOCI excl. TMICC 561 (2,216 - 1,655) + non-current FVTPL 'Other' 341 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) p.174 note 17A); amortised-cost assets 368 (incl. judicial deposits 175) excluded; (5) net Magnum transition balance owed to Unilever 2,100 - 1,600 = 500 (Unilever FY25 Form 20-F (SEC accession 0000217410-26-000007, filed 12 Mar 2026, https://www.sec.gov/Archives/edgar/data/217410/000021741026000007/ul-20251231.htm) notes 13-14, p.159-160). Was 2,044.2 (TMICC + JVs/associates at book 109). If the run's cost of equity changes, the JV value must be recomputed. JV value recomputed 15 Oct 2026 at the new cost of equity 7.1645% (ERP 4.2%): 229 x 1.016 / (7.1645% - 1.6%) = 4181.2 (was 3709.6 at 7.8720%)</t>
         </is>
       </c>
     </row>
@@ -839,11 +839,11 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>33955.3</v>
+        <v>33312.4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Foods consideration at run-date market value (decision 1): cash USD 15,700m + new McCormick shares 499,691,175 (= existing 269,064,479 [voting 14,522,864 + non-voting 254,541,615, McCormick 10-Q for the quarter to 31 Aug 2026 (accession 0000063754-26-000329, filed 1 Oct 2026, https://www.sec.gov/Archives/edgar/data/63754/000006375426000329/mkc-20260831.htm) cover] x 65/35; 55.1% to Unilever shareholders + 9.9% to Unilever, 10-Q note 2) x USD 44.64 (Yahoo MKC close 2026-10-13) = USD 22,306.2m; total USD 38,006.2m / 1.1193 USD per EUR (FRED DEXUSEU 2026-10-09) = EUR 33,955.3m. Yahoo EURUSD=X 1.1160 (2026-10-12) would give 34,055.1. Tax on the cash: MISSING, NOT deducted (PM decision 5; CFO: 'premature to start making estimates', Unilever investor call transcript 31 Mar 2026, Form 425 (accession 0000217410-26-000032)). Received at closing (expected mid-2027): timing FLAG in notes.md.</t>
+          <t>Foods consideration at run-date market value (decision 1): cash USD 15,700m + new McCormick shares 499,691,175 (= existing 269,064,479 [voting 14,522,864 + non-voting 254,541,615, McCormick 10-Q for the quarter to 31 Aug 2026 (accession 0000063754-26-000329, filed 1 Oct 2026, https://www.sec.gov/Archives/edgar/data/63754/000006375426000329/mkc-20260831.htm) cover] x 65/35; 55.1% to Unilever shareholders + 9.9% to Unilever, 10-Q note 2) x USD 44.64 (Yahoo MKC close 2026-10-13) = USD 22,306.2m; total USD 38,006.2m / 1.1193 USD per EUR (FRED DEXUSEU 2026-10-09) = EUR 33,955.3m. Yahoo EURUSD=X 1.1160 (2026-10-12) would give 34,055.1. Tax on the cash: MISSING, NOT deducted (PM decision 5; CFO: 'premature to start making estimates', Unilever investor call transcript 31 Mar 2026, Form 425 (accession 0000217410-26-000032)). Received at closing (expected mid-2027): timing FLAG in notes.md. LESS McCormick dividends the new shares miss before closing (PM decision 15 Oct 2026): 499,691,175 shares x USD 0.48 a quarter (McCormick 10-Q to 31 Aug 2026, accession 0000063754-26-000329) x 3 quarters (ex-dates Jan, Apr, Jul 2027; closing expected mid-2027, Form 425 0000217410-26-000027) / 1.1193 USD per EUR (FRED DEXUSEU 2026-10-09) = 642.9; 33955.3 - 642.9. FLAG: if closing comes before the July ex-date, 2 quarters (+c.8p)</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.005</v>
+        <v>0.02</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0.016</v>
@@ -1035,7 +1035,7 @@
         <v/>
       </c>
       <c r="I3" s="4" t="n">
-        <v>42624.24506962581</v>
+        <v>43260.42783185904</v>
       </c>
     </row>
     <row r="4">
@@ -1092,7 +1092,7 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>7544.491377323768</v>
+        <v>7657.095726239049</v>
       </c>
     </row>
     <row r="6">
@@ -1257,7 +1257,7 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>5428.899063728622</v>
+        <v>5509.927407963378</v>
       </c>
     </row>
     <row r="12">
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>3987.561070822048</v>
+        <v>4149.533706350344</v>
       </c>
     </row>
     <row r="16">
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.07872000000000001</v>
+        <v>0.07164480000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1422,7 +1422,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.0709735865</v>
+        <v>0.06503997002</v>
       </c>
     </row>
     <row r="20">
@@ -1436,7 +1436,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>22165.44187139205</v>
+        <v>22867.77215716328</v>
       </c>
     </row>
     <row r="21">
@@ -1450,7 +1450,7 @@
         <v/>
       </c>
       <c r="C21" s="4" t="n">
-        <v>5162.385192890956</v>
+        <v>5239.435718157987</v>
       </c>
     </row>
     <row r="22">
@@ -1464,7 +1464,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>93906.64720212416</v>
+        <v>106840.1085078393</v>
       </c>
     </row>
     <row r="23">
@@ -1478,7 +1478,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>68975.03274216867</v>
+        <v>80461.42873001605</v>
       </c>
     </row>
     <row r="24">
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>91140.47461356071</v>
+        <v>103329.2008871793</v>
       </c>
     </row>
     <row r="25">
@@ -1506,7 +1506,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>9737.448307712826</v>
+        <v>11039.69182278624</v>
       </c>
     </row>
     <row r="26">
@@ -1520,7 +1520,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>98844.12630584789</v>
+        <v>108860.8090643931</v>
       </c>
     </row>
     <row r="27">
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>98163.22535806705</v>
+        <v>108431.0974823262</v>
       </c>
     </row>
     <row r="28">
@@ -1548,7 +1548,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>45.56559754476966</v>
+        <v>50.33175846856314</v>
       </c>
     </row>
     <row r="29">
@@ -1562,7 +1562,7 @@
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3855.285609786128</v>
+        <v>4258.548435547867</v>
       </c>
     </row>
     <row r="30">
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>-0.1815549072</v>
+        <v>-0.0959455609</v>
       </c>
     </row>
   </sheetData>

</xml_diff>